<commit_message>
adionei validações e alterei o requerimento.md
</commit_message>
<xml_diff>
--- a/quentinha.xlsx
+++ b/quentinha.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,47 +432,29 @@
           <t>Valor Devedor</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>total</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>wil</t>
+          <t>wilson</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="C2" t="n">
-        <v>336</v>
+        <v>32</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>qq</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>44</v>
-      </c>
-      <c r="C3" t="n">
-        <v>704</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
+    <row r="4">
+      <c r="A4" t="inlineStr">
         <is>
           <t>TOTAL GERAL</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
-      <c r="C5" t="n">
-        <v>1040</v>
+      <c r="B4" t="inlineStr"/>
+      <c r="C4" t="n">
+        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>